<commit_message>
Sync with code with pitch repository
</commit_message>
<xml_diff>
--- a/BaseScenarios.xlsx
+++ b/BaseScenarios.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tmt/Library/CloudStorage/Dropbox/UCA/Intro-Software-Engineering/source/pitch/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tmt/Library/CloudStorage/Dropbox/UCA/Intro-Software-Engineering/source/pitch_student/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{870CD2EC-B2E4-4A48-9DEF-395D13A20EBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{734FE8A3-547A-474F-8DFE-C103A13075DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-42660" yWindow="-13240" windowWidth="39940" windowHeight="15660" xr2:uid="{A28C8302-46F6-CF46-ACCA-48740F3E371A}"/>
+    <workbookView xWindow="-42660" yWindow="-13240" windowWidth="39940" windowHeight="15660" activeTab="1" xr2:uid="{A28C8302-46F6-CF46-ACCA-48740F3E371A}"/>
   </bookViews>
   <sheets>
-    <sheet name="Position_1" sheetId="4" r:id="rId1"/>
-    <sheet name="Position_2" sheetId="5" r:id="rId2"/>
-    <sheet name="Position_3" sheetId="6" r:id="rId3"/>
-    <sheet name="Position_4" sheetId="7" r:id="rId4"/>
-    <sheet name="standard_bid" sheetId="8" r:id="rId5"/>
-    <sheet name="aggressive_bid" sheetId="9" r:id="rId6"/>
+    <sheet name="standard_bid" sheetId="8" r:id="rId1"/>
+    <sheet name="aggressive_bid" sheetId="9" r:id="rId2"/>
+    <sheet name="Position_1" sheetId="4" r:id="rId3"/>
+    <sheet name="Position_2" sheetId="5" r:id="rId4"/>
+    <sheet name="Position_3" sheetId="6" r:id="rId5"/>
+    <sheet name="Position_4" sheetId="7" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -180,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -213,12 +213,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -552,6 +546,330 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FF63575-79E1-FD42-8E26-375EF79FFFF1}">
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>17</v>
+      </c>
+      <c r="B2" s="11">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>16</v>
+      </c>
+      <c r="B3" s="11">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>15</v>
+      </c>
+      <c r="B4" s="11">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>14</v>
+      </c>
+      <c r="B5" s="11">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>13</v>
+      </c>
+      <c r="B6" s="11">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>12</v>
+      </c>
+      <c r="B7" s="11">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>11</v>
+      </c>
+      <c r="B8" s="11">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>10</v>
+      </c>
+      <c r="B9" s="11">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="11">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>8</v>
+      </c>
+      <c r="B11" s="11">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>7</v>
+      </c>
+      <c r="B12" s="11">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>6</v>
+      </c>
+      <c r="B13" s="11">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>5</v>
+      </c>
+      <c r="B14" s="11">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>4</v>
+      </c>
+      <c r="B15" s="11">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>3</v>
+      </c>
+      <c r="B16" s="11">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>2</v>
+      </c>
+      <c r="B17" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>1</v>
+      </c>
+      <c r="B18" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>0</v>
+      </c>
+      <c r="B19" s="11">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16516A00-C0F0-E64D-A560-E6FE8524E6EA}">
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>17</v>
+      </c>
+      <c r="B2" s="11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>16</v>
+      </c>
+      <c r="B3" s="11">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>15</v>
+      </c>
+      <c r="B4" s="11">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>14</v>
+      </c>
+      <c r="B5" s="11">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>13</v>
+      </c>
+      <c r="B6" s="11">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>12</v>
+      </c>
+      <c r="B7" s="11">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>11</v>
+      </c>
+      <c r="B8" s="11">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>10</v>
+      </c>
+      <c r="B9" s="11">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="11">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>8</v>
+      </c>
+      <c r="B11" s="11">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>7</v>
+      </c>
+      <c r="B12" s="11">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>6</v>
+      </c>
+      <c r="B13" s="11">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>5</v>
+      </c>
+      <c r="B14" s="11">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>4</v>
+      </c>
+      <c r="B15" s="11">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>3</v>
+      </c>
+      <c r="B16" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>2</v>
+      </c>
+      <c r="B17" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>1</v>
+      </c>
+      <c r="B18" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>0</v>
+      </c>
+      <c r="B19" s="11">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A07370E1-2B8D-004C-84E7-79A5F5CF6E30}">
   <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -827,7 +1145,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{850E1FFC-8612-3E43-B5A8-44C12DE068D4}">
   <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1018,7 +1336,7 @@
       <c r="L6" s="5"/>
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
-      <c r="O6" s="12"/>
+      <c r="O6" s="1"/>
       <c r="P6" s="1"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
@@ -1036,7 +1354,7 @@
       <c r="L7" s="5"/>
       <c r="M7" s="5"/>
       <c r="N7" s="5"/>
-      <c r="O7" s="12"/>
+      <c r="O7" s="1"/>
       <c r="P7" s="1"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
@@ -1077,7 +1395,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C0F7248-492C-FE4F-A9CD-2C693D2FEAB9}">
   <dimension ref="A1:P15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1557,14 +1875,14 @@
       <c r="O15" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="P15" s="12"/>
+      <c r="P15" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C6593C9-3805-8045-9BFF-AD45268F99A4}">
   <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1879,8 +2197,8 @@
       <c r="L10" s="7"/>
       <c r="M10" s="7"/>
       <c r="N10" s="7"/>
-      <c r="O10" s="12"/>
-      <c r="P10" s="13"/>
+      <c r="O10" s="1"/>
+      <c r="P10" s="8"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="G11" s="5"/>
@@ -1899,330 +2217,6 @@
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="G16" s="5"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FF63575-79E1-FD42-8E26-375EF79FFFF1}">
-  <dimension ref="A1:B19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>17</v>
-      </c>
-      <c r="B2" s="11">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>16</v>
-      </c>
-      <c r="B3" s="11">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>15</v>
-      </c>
-      <c r="B4" s="11">
-        <v>1.25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>14</v>
-      </c>
-      <c r="B5" s="11">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>13</v>
-      </c>
-      <c r="B6" s="11">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>12</v>
-      </c>
-      <c r="B7" s="11">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>11</v>
-      </c>
-      <c r="B8" s="11">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>10</v>
-      </c>
-      <c r="B9" s="11">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" s="11">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11">
-        <v>8</v>
-      </c>
-      <c r="B11" s="11">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12">
-        <v>7</v>
-      </c>
-      <c r="B12" s="11">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>6</v>
-      </c>
-      <c r="B13" s="11">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14">
-        <v>5</v>
-      </c>
-      <c r="B14" s="11">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A15">
-        <v>4</v>
-      </c>
-      <c r="B15" s="11">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16">
-        <v>3</v>
-      </c>
-      <c r="B16" s="11">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17">
-        <v>2</v>
-      </c>
-      <c r="B17" s="11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18">
-        <v>1</v>
-      </c>
-      <c r="B18" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19">
-        <v>0</v>
-      </c>
-      <c r="B19" s="11">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16516A00-C0F0-E64D-A560-E6FE8524E6EA}">
-  <dimension ref="A1:B19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>17</v>
-      </c>
-      <c r="B2" s="11">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>16</v>
-      </c>
-      <c r="B3" s="11">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>15</v>
-      </c>
-      <c r="B4" s="11">
-        <v>1.25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>14</v>
-      </c>
-      <c r="B5" s="11">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>13</v>
-      </c>
-      <c r="B6" s="11">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>12</v>
-      </c>
-      <c r="B7" s="11">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>11</v>
-      </c>
-      <c r="B8" s="11">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>10</v>
-      </c>
-      <c r="B9" s="11">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" s="11">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11">
-        <v>8</v>
-      </c>
-      <c r="B11" s="11">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12">
-        <v>7</v>
-      </c>
-      <c r="B12" s="11">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>6</v>
-      </c>
-      <c r="B13" s="11">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14">
-        <v>5</v>
-      </c>
-      <c r="B14" s="11">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A15">
-        <v>4</v>
-      </c>
-      <c r="B15" s="11">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16">
-        <v>3</v>
-      </c>
-      <c r="B16" s="11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17">
-        <v>2</v>
-      </c>
-      <c r="B17" s="11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18">
-        <v>1</v>
-      </c>
-      <c r="B18" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19">
-        <v>0</v>
-      </c>
-      <c r="B19" s="11">
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>